<commit_message>
docs(anexos): renomeia MARIA->MARIAH e nome por extenso nos documentos de public/
</commit_message>
<xml_diff>
--- a/public/planilha-validacao-local-maria.xlsx
+++ b/public/planilha-validacao-local-maria.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="104">
   <si>
-    <t xml:space="preserve">Planilha-modelo · Apêndice F · Validação Local da MARIA pelos CEPs</t>
+    <t xml:space="preserve">Planilha-modelo · Apêndice F · Validação Local da MARIAH pelos CEPs</t>
   </si>
   <si>
     <t xml:space="preserve">Esta planilha automatiza o registro e o cálculo dos indicadores das três frentes de validação propostas no Apêndice F. Use-a no Microsoft Excel, no LibreOffice Calc ou no Google Sheets — não requer instalação de extensão estatística.</t>
@@ -267,7 +267,7 @@
     <t xml:space="preserve">Painel-resumo das três frentes de validação</t>
   </si>
   <si>
-    <t xml:space="preserve">Este painel consolida os indicadores das três frentes. Use-o como ponto de partida da reunião plenária do CEP que discutir os achados da validação local da MARIA. CEPs que optarem por compartilhar resultados com o Grupo de Trabalho podem enviar somente este painel, sem prejuízo de detalhamento posterior.</t>
+    <t xml:space="preserve">Este painel consolida os indicadores das três frentes. Use-o como ponto de partida da reunião plenária do CEP que discutir os achados da validação local da MARIAH. CEPs que optarem por compartilhar resultados com o Grupo de Trabalho podem enviar somente este painel, sem prejuízo de detalhamento posterior.</t>
   </si>
   <si>
     <t xml:space="preserve">Frente 1 — Concordância entre avaliadores na Versão A</t>

</xml_diff>